<commit_message>
update bill page -5333945704
</commit_message>
<xml_diff>
--- a/bills/JXZFSP01/-5333945704/a17b74460300c96f2383c5c7d4608f5756166fa0853565f47ff5d014fb4ede3a/bill-2026-09-10.xlsx
+++ b/bills/JXZFSP01/-5333945704/a17b74460300c96f2383c5c7d4608f5756166fa0853565f47ff5d014fb4ede3a/bill-2026-09-10.xlsx
@@ -199,59 +199,86 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>总计</t>
-        </is>
-      </c>
-    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>09/10 18:54:57</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>xinhui9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>总入款</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>90000</t>
+          <t>总计</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>应下发</t>
+          <t>总入款</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>9782.61</t>
+          <t>90000</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>已下发</t>
+          <t>应下发</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9782.61</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>已下发</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>未下发</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>9782.61</t>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>8894.61</t>
         </is>
       </c>
     </row>

</xml_diff>